<commit_message>
queda pendent seguir i treballar els duplicats de live
</commit_message>
<xml_diff>
--- a/WG specific variables_final_202604.xlsx
+++ b/WG specific variables_final_202604.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\management\Data_Documentation\Data_management\Endpoints\Working Groups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\Diccionari-IARC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE226669-6945-48D4-AF24-7DD512C62CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F18AA10E-D2DC-4F39-BC7F-48B180F405CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C816575C-BAC2-4178-A389-3D7121D8EAF4}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C816575C-BAC2-4178-A389-3D7121D8EAF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Wg specific variables " sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wg specific variables '!$A$1:$F$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1472,6 +1475,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1481,47 +1525,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1540,7 +1543,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1857,7 +1860,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E11F5BF0-69CA-44BB-85F3-E3ED603EB111}">
   <dimension ref="A1:F145"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -1924,13 +1927,13 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="55" t="s">
+      <c r="A4" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="64" t="s">
+      <c r="C4" s="61" t="s">
         <v>118</v>
       </c>
       <c r="D4" s="14" t="s">
@@ -1942,9 +1945,9 @@
       <c r="F4" s="37"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="56"/>
-      <c r="B5" s="56"/>
-      <c r="C5" s="64"/>
+      <c r="A5" s="71"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="61"/>
       <c r="D5" s="14" t="s">
         <v>8</v>
       </c>
@@ -1954,9 +1957,9 @@
       <c r="F5" s="38"/>
     </row>
     <row r="6" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="56"/>
-      <c r="B6" s="56"/>
-      <c r="C6" s="64"/>
+      <c r="A6" s="71"/>
+      <c r="B6" s="71"/>
+      <c r="C6" s="61"/>
       <c r="D6" s="14" t="s">
         <v>9</v>
       </c>
@@ -1966,9 +1969,9 @@
       <c r="F6" s="38"/>
     </row>
     <row r="7" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="56"/>
-      <c r="B7" s="56"/>
-      <c r="C7" s="64"/>
+      <c r="A7" s="71"/>
+      <c r="B7" s="71"/>
+      <c r="C7" s="61"/>
       <c r="D7" s="14" t="s">
         <v>10</v>
       </c>
@@ -1978,9 +1981,9 @@
       <c r="F7" s="38"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="56"/>
-      <c r="B8" s="56"/>
-      <c r="C8" s="64"/>
+      <c r="A8" s="71"/>
+      <c r="B8" s="71"/>
+      <c r="C8" s="61"/>
       <c r="D8" s="14" t="s">
         <v>11</v>
       </c>
@@ -1990,9 +1993,9 @@
       <c r="F8" s="38"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="56"/>
-      <c r="B9" s="56"/>
-      <c r="C9" s="64"/>
+      <c r="A9" s="71"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="61"/>
       <c r="D9" s="14" t="s">
         <v>12</v>
       </c>
@@ -2004,9 +2007,9 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="56"/>
-      <c r="B10" s="56"/>
-      <c r="C10" s="64"/>
+      <c r="A10" s="71"/>
+      <c r="B10" s="71"/>
+      <c r="C10" s="61"/>
       <c r="D10" s="14" t="s">
         <v>13</v>
       </c>
@@ -2018,9 +2021,9 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="56"/>
-      <c r="B11" s="56"/>
-      <c r="C11" s="64"/>
+      <c r="A11" s="71"/>
+      <c r="B11" s="71"/>
+      <c r="C11" s="61"/>
       <c r="D11" s="14" t="s">
         <v>14</v>
       </c>
@@ -2032,9 +2035,9 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="56"/>
-      <c r="B12" s="56"/>
-      <c r="C12" s="64"/>
+      <c r="A12" s="71"/>
+      <c r="B12" s="71"/>
+      <c r="C12" s="61"/>
       <c r="D12" s="14" t="s">
         <v>15</v>
       </c>
@@ -2046,9 +2049,9 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="57"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="65"/>
+      <c r="A13" s="72"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="62"/>
       <c r="D13" s="15" t="s">
         <v>16</v>
       </c>
@@ -2060,10 +2063,10 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="55" t="s">
+      <c r="A14" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="70" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="63" t="s">
@@ -2078,9 +2081,9 @@
       <c r="F14" s="37"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="56"/>
-      <c r="B15" s="56"/>
-      <c r="C15" s="64"/>
+      <c r="A15" s="71"/>
+      <c r="B15" s="71"/>
+      <c r="C15" s="61"/>
       <c r="D15" s="14" t="s">
         <v>20</v>
       </c>
@@ -2090,9 +2093,9 @@
       <c r="F15" s="38"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="56"/>
-      <c r="B16" s="56"/>
-      <c r="C16" s="64"/>
+      <c r="A16" s="71"/>
+      <c r="B16" s="71"/>
+      <c r="C16" s="61"/>
       <c r="D16" s="14" t="s">
         <v>21</v>
       </c>
@@ -2102,9 +2105,9 @@
       <c r="F16" s="38"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="56"/>
-      <c r="B17" s="56"/>
-      <c r="C17" s="64"/>
+      <c r="A17" s="71"/>
+      <c r="B17" s="71"/>
+      <c r="C17" s="61"/>
       <c r="D17" s="14" t="s">
         <v>22</v>
       </c>
@@ -2114,9 +2117,9 @@
       <c r="F17" s="38"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="57"/>
-      <c r="B18" s="57"/>
-      <c r="C18" s="65"/>
+      <c r="A18" s="72"/>
+      <c r="B18" s="72"/>
+      <c r="C18" s="62"/>
       <c r="D18" s="15" t="s">
         <v>23</v>
       </c>
@@ -2126,10 +2129,10 @@
       <c r="F18" s="38"/>
     </row>
     <row r="19" spans="1:6" ht="51" x14ac:dyDescent="0.25">
-      <c r="A19" s="55" t="s">
+      <c r="A19" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="55" t="s">
+      <c r="B19" s="70" t="s">
         <v>25</v>
       </c>
       <c r="C19" s="63" t="s">
@@ -2144,9 +2147,9 @@
       <c r="F19" s="37"/>
     </row>
     <row r="20" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="56"/>
-      <c r="B20" s="56"/>
-      <c r="C20" s="64"/>
+      <c r="A20" s="71"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="61"/>
       <c r="D20" s="14" t="s">
         <v>246</v>
       </c>
@@ -2157,10 +2160,10 @@
         <v>317</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="56"/>
-      <c r="B21" s="56"/>
-      <c r="C21" s="64"/>
+    <row r="21" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="71"/>
+      <c r="B21" s="71"/>
+      <c r="C21" s="61"/>
       <c r="D21" s="14" t="s">
         <v>247</v>
       </c>
@@ -2170,9 +2173,9 @@
       <c r="F21" s="38"/>
     </row>
     <row r="22" spans="1:6" ht="153" x14ac:dyDescent="0.25">
-      <c r="A22" s="56"/>
-      <c r="B22" s="56"/>
-      <c r="C22" s="64"/>
+      <c r="A22" s="71"/>
+      <c r="B22" s="71"/>
+      <c r="C22" s="61"/>
       <c r="D22" s="14" t="s">
         <v>248</v>
       </c>
@@ -2182,9 +2185,9 @@
       <c r="F22" s="38"/>
     </row>
     <row r="23" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A23" s="56"/>
-      <c r="B23" s="56"/>
-      <c r="C23" s="64"/>
+      <c r="A23" s="71"/>
+      <c r="B23" s="71"/>
+      <c r="C23" s="61"/>
       <c r="D23" s="14" t="s">
         <v>249</v>
       </c>
@@ -2194,9 +2197,9 @@
       <c r="F23" s="38"/>
     </row>
     <row r="24" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="56"/>
-      <c r="B24" s="56"/>
-      <c r="C24" s="64"/>
+      <c r="A24" s="71"/>
+      <c r="B24" s="71"/>
+      <c r="C24" s="61"/>
       <c r="D24" s="14" t="s">
         <v>250</v>
       </c>
@@ -2206,9 +2209,9 @@
       <c r="F24" s="38"/>
     </row>
     <row r="25" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A25" s="56"/>
-      <c r="B25" s="56"/>
-      <c r="C25" s="64"/>
+      <c r="A25" s="71"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="61"/>
       <c r="D25" s="14" t="s">
         <v>251</v>
       </c>
@@ -2218,9 +2221,9 @@
       <c r="F25" s="38"/>
     </row>
     <row r="26" spans="1:6" ht="51" x14ac:dyDescent="0.25">
-      <c r="A26" s="56"/>
-      <c r="B26" s="56"/>
-      <c r="C26" s="64"/>
+      <c r="A26" s="71"/>
+      <c r="B26" s="71"/>
+      <c r="C26" s="61"/>
       <c r="D26" s="14" t="s">
         <v>252</v>
       </c>
@@ -2230,9 +2233,9 @@
       <c r="F26" s="38"/>
     </row>
     <row r="27" spans="1:6" ht="127.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="56"/>
-      <c r="B27" s="56"/>
-      <c r="C27" s="64"/>
+      <c r="A27" s="71"/>
+      <c r="B27" s="71"/>
+      <c r="C27" s="61"/>
       <c r="D27" s="14" t="s">
         <v>253</v>
       </c>
@@ -2242,9 +2245,9 @@
       <c r="F27" s="38"/>
     </row>
     <row r="28" spans="1:6" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="56"/>
-      <c r="B28" s="56"/>
-      <c r="C28" s="64"/>
+      <c r="A28" s="71"/>
+      <c r="B28" s="71"/>
+      <c r="C28" s="61"/>
       <c r="D28" s="14" t="s">
         <v>285</v>
       </c>
@@ -2256,9 +2259,9 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="102" x14ac:dyDescent="0.25">
-      <c r="A29" s="56"/>
-      <c r="B29" s="56"/>
-      <c r="C29" s="64"/>
+      <c r="A29" s="71"/>
+      <c r="B29" s="71"/>
+      <c r="C29" s="61"/>
       <c r="D29" s="14" t="s">
         <v>286</v>
       </c>
@@ -2270,9 +2273,9 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="56"/>
-      <c r="B30" s="56"/>
-      <c r="C30" s="64"/>
+      <c r="A30" s="71"/>
+      <c r="B30" s="71"/>
+      <c r="C30" s="61"/>
       <c r="D30" s="14" t="s">
         <v>265</v>
       </c>
@@ -2282,9 +2285,9 @@
       <c r="F30" s="38"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="56"/>
-      <c r="B31" s="56"/>
-      <c r="C31" s="64"/>
+      <c r="A31" s="71"/>
+      <c r="B31" s="71"/>
+      <c r="C31" s="61"/>
       <c r="D31" s="14" t="s">
         <v>284</v>
       </c>
@@ -2294,9 +2297,9 @@
       <c r="F31" s="53"/>
     </row>
     <row r="32" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="57"/>
-      <c r="B32" s="56"/>
-      <c r="C32" s="65"/>
+      <c r="A32" s="72"/>
+      <c r="B32" s="71"/>
+      <c r="C32" s="62"/>
       <c r="D32" s="15" t="s">
         <v>254</v>
       </c>
@@ -2345,7 +2348,7 @@
       <c r="A35" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B35" s="58" t="s">
+      <c r="B35" s="67" t="s">
         <v>30</v>
       </c>
       <c r="C35" s="63" t="s">
@@ -2360,9 +2363,9 @@
       <c r="F35" s="37"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="64"/>
-      <c r="B36" s="59"/>
-      <c r="C36" s="64"/>
+      <c r="A36" s="61"/>
+      <c r="B36" s="68"/>
+      <c r="C36" s="61"/>
       <c r="D36" s="29" t="s">
         <v>95</v>
       </c>
@@ -2372,9 +2375,9 @@
       <c r="F36" s="38"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="64"/>
-      <c r="B37" s="59"/>
-      <c r="C37" s="64"/>
+      <c r="A37" s="61"/>
+      <c r="B37" s="68"/>
+      <c r="C37" s="61"/>
       <c r="D37" s="29" t="s">
         <v>96</v>
       </c>
@@ -2384,9 +2387,9 @@
       <c r="F37" s="38"/>
     </row>
     <row r="38" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A38" s="64"/>
-      <c r="B38" s="59"/>
-      <c r="C38" s="64"/>
+      <c r="A38" s="61"/>
+      <c r="B38" s="68"/>
+      <c r="C38" s="61"/>
       <c r="D38" s="29" t="s">
         <v>97</v>
       </c>
@@ -2396,9 +2399,9 @@
       <c r="F38" s="38"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="64"/>
-      <c r="B39" s="59"/>
-      <c r="C39" s="64"/>
+      <c r="A39" s="61"/>
+      <c r="B39" s="68"/>
+      <c r="C39" s="61"/>
       <c r="D39" s="29" t="s">
         <v>98</v>
       </c>
@@ -2408,9 +2411,9 @@
       <c r="F39" s="38"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="64"/>
-      <c r="B40" s="59"/>
-      <c r="C40" s="64"/>
+      <c r="A40" s="61"/>
+      <c r="B40" s="68"/>
+      <c r="C40" s="61"/>
       <c r="D40" s="29" t="s">
         <v>99</v>
       </c>
@@ -2420,9 +2423,9 @@
       <c r="F40" s="38"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="64"/>
-      <c r="B41" s="59"/>
-      <c r="C41" s="64"/>
+      <c r="A41" s="61"/>
+      <c r="B41" s="68"/>
+      <c r="C41" s="61"/>
       <c r="D41" s="29" t="s">
         <v>100</v>
       </c>
@@ -2432,9 +2435,9 @@
       <c r="F41" s="38"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="64"/>
-      <c r="B42" s="59"/>
-      <c r="C42" s="64"/>
+      <c r="A42" s="61"/>
+      <c r="B42" s="68"/>
+      <c r="C42" s="61"/>
       <c r="D42" s="29" t="s">
         <v>101</v>
       </c>
@@ -2444,9 +2447,9 @@
       <c r="F42" s="38"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="64"/>
-      <c r="B43" s="59"/>
-      <c r="C43" s="64"/>
+      <c r="A43" s="61"/>
+      <c r="B43" s="68"/>
+      <c r="C43" s="61"/>
       <c r="D43" s="40" t="s">
         <v>102</v>
       </c>
@@ -2456,9 +2459,9 @@
       <c r="F43" s="38"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="64"/>
-      <c r="B44" s="59"/>
-      <c r="C44" s="64"/>
+      <c r="A44" s="61"/>
+      <c r="B44" s="68"/>
+      <c r="C44" s="61"/>
       <c r="D44" s="40" t="s">
         <v>103</v>
       </c>
@@ -2468,9 +2471,9 @@
       <c r="F44" s="38"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="64"/>
-      <c r="B45" s="59"/>
-      <c r="C45" s="64"/>
+      <c r="A45" s="61"/>
+      <c r="B45" s="68"/>
+      <c r="C45" s="61"/>
       <c r="D45" s="40" t="s">
         <v>104</v>
       </c>
@@ -2480,9 +2483,9 @@
       <c r="F45" s="38"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="64"/>
-      <c r="B46" s="59"/>
-      <c r="C46" s="64"/>
+      <c r="A46" s="61"/>
+      <c r="B46" s="68"/>
+      <c r="C46" s="61"/>
       <c r="D46" s="40" t="s">
         <v>105</v>
       </c>
@@ -2492,9 +2495,9 @@
       <c r="F46" s="38"/>
     </row>
     <row r="47" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="64"/>
-      <c r="B47" s="59"/>
-      <c r="C47" s="64"/>
+      <c r="A47" s="61"/>
+      <c r="B47" s="68"/>
+      <c r="C47" s="61"/>
       <c r="D47" s="40" t="s">
         <v>106</v>
       </c>
@@ -2504,9 +2507,9 @@
       <c r="F47" s="38"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="64"/>
-      <c r="B48" s="59"/>
-      <c r="C48" s="64"/>
+      <c r="A48" s="61"/>
+      <c r="B48" s="68"/>
+      <c r="C48" s="61"/>
       <c r="D48" s="40" t="s">
         <v>116</v>
       </c>
@@ -2516,9 +2519,9 @@
       <c r="F48" s="38"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="64"/>
-      <c r="B49" s="59"/>
-      <c r="C49" s="64"/>
+      <c r="A49" s="61"/>
+      <c r="B49" s="68"/>
+      <c r="C49" s="61"/>
       <c r="D49" s="40" t="s">
         <v>107</v>
       </c>
@@ -2530,9 +2533,9 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="64"/>
-      <c r="B50" s="59"/>
-      <c r="C50" s="64"/>
+      <c r="A50" s="61"/>
+      <c r="B50" s="68"/>
+      <c r="C50" s="61"/>
       <c r="D50" s="40" t="s">
         <v>108</v>
       </c>
@@ -2544,9 +2547,9 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="65"/>
-      <c r="B51" s="60"/>
-      <c r="C51" s="65"/>
+      <c r="A51" s="62"/>
+      <c r="B51" s="69"/>
+      <c r="C51" s="62"/>
       <c r="D51" s="41" t="s">
         <v>109</v>
       </c>
@@ -2558,27 +2561,27 @@
       </c>
     </row>
     <row r="52" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="55" t="s">
+      <c r="A52" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="B52" s="56" t="s">
+      <c r="B52" s="71" t="s">
         <v>32</v>
       </c>
       <c r="C52" s="63" t="s">
         <v>124</v>
       </c>
-      <c r="D52" s="68" t="s">
+      <c r="D52" s="55" t="s">
         <v>33</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="F52" s="71"/>
+      <c r="F52" s="58"/>
     </row>
     <row r="53" spans="1:6" ht="102" x14ac:dyDescent="0.25">
-      <c r="A53" s="56"/>
-      <c r="B53" s="56"/>
-      <c r="C53" s="64"/>
+      <c r="A53" s="71"/>
+      <c r="B53" s="71"/>
+      <c r="C53" s="61"/>
       <c r="D53" s="34" t="s">
         <v>110</v>
       </c>
@@ -2588,10 +2591,10 @@
       <c r="F53" s="42"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="56"/>
-      <c r="B54" s="56"/>
-      <c r="C54" s="64"/>
-      <c r="D54" s="69" t="s">
+      <c r="A54" s="71"/>
+      <c r="B54" s="71"/>
+      <c r="C54" s="61"/>
+      <c r="D54" s="56" t="s">
         <v>111</v>
       </c>
       <c r="E54" s="1" t="s">
@@ -2600,9 +2603,9 @@
       <c r="F54" s="42"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="56"/>
-      <c r="B55" s="56"/>
-      <c r="C55" s="64"/>
+      <c r="A55" s="71"/>
+      <c r="B55" s="71"/>
+      <c r="C55" s="61"/>
       <c r="D55" s="34" t="s">
         <v>113</v>
       </c>
@@ -2612,9 +2615,9 @@
       <c r="F55" s="42"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="56"/>
-      <c r="B56" s="56"/>
-      <c r="C56" s="64"/>
+      <c r="A56" s="71"/>
+      <c r="B56" s="71"/>
+      <c r="C56" s="61"/>
       <c r="D56" s="34" t="s">
         <v>112</v>
       </c>
@@ -2624,9 +2627,9 @@
       <c r="F56" s="42"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="56"/>
-      <c r="B57" s="56"/>
-      <c r="C57" s="64"/>
+      <c r="A57" s="71"/>
+      <c r="B57" s="71"/>
+      <c r="C57" s="61"/>
       <c r="D57" s="34" t="s">
         <v>114</v>
       </c>
@@ -2636,9 +2639,9 @@
       <c r="F57" s="42"/>
     </row>
     <row r="58" spans="1:6" ht="102" x14ac:dyDescent="0.25">
-      <c r="A58" s="56"/>
-      <c r="B58" s="56"/>
-      <c r="C58" s="64"/>
+      <c r="A58" s="71"/>
+      <c r="B58" s="71"/>
+      <c r="C58" s="61"/>
       <c r="D58" s="34" t="s">
         <v>115</v>
       </c>
@@ -2648,9 +2651,9 @@
       <c r="F58" s="42"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="56"/>
-      <c r="B59" s="56"/>
-      <c r="C59" s="64"/>
+      <c r="A59" s="71"/>
+      <c r="B59" s="71"/>
+      <c r="C59" s="61"/>
       <c r="D59" s="34" t="s">
         <v>106</v>
       </c>
@@ -2660,9 +2663,9 @@
       <c r="F59" s="42"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="56"/>
-      <c r="B60" s="56"/>
-      <c r="C60" s="64"/>
+      <c r="A60" s="71"/>
+      <c r="B60" s="71"/>
+      <c r="C60" s="61"/>
       <c r="D60" s="34" t="s">
         <v>105</v>
       </c>
@@ -2672,22 +2675,22 @@
       <c r="F60" s="42"/>
     </row>
     <row r="61" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="57"/>
-      <c r="B61" s="57"/>
-      <c r="C61" s="65"/>
-      <c r="D61" s="70" t="s">
+      <c r="A61" s="72"/>
+      <c r="B61" s="72"/>
+      <c r="C61" s="62"/>
+      <c r="D61" s="57" t="s">
         <v>116</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="F61" s="72"/>
+      <c r="F61" s="59"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="55" t="s">
+      <c r="A62" s="70" t="s">
         <v>34</v>
       </c>
-      <c r="B62" s="55" t="s">
+      <c r="B62" s="70" t="s">
         <v>35</v>
       </c>
       <c r="C62" s="63" t="s">
@@ -2702,9 +2705,9 @@
       <c r="F62" s="42"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="56"/>
-      <c r="B63" s="56"/>
-      <c r="C63" s="64"/>
+      <c r="A63" s="71"/>
+      <c r="B63" s="71"/>
+      <c r="C63" s="61"/>
       <c r="D63" s="14" t="s">
         <v>37</v>
       </c>
@@ -2714,9 +2717,9 @@
       <c r="F63" s="42"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="56"/>
-      <c r="B64" s="56"/>
-      <c r="C64" s="64"/>
+      <c r="A64" s="71"/>
+      <c r="B64" s="71"/>
+      <c r="C64" s="61"/>
       <c r="D64" s="14" t="s">
         <v>140</v>
       </c>
@@ -2725,10 +2728,10 @@
       </c>
       <c r="F64" s="42"/>
     </row>
-    <row r="65" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="56"/>
-      <c r="B65" s="56"/>
-      <c r="C65" s="64"/>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="71"/>
+      <c r="B65" s="71"/>
+      <c r="C65" s="61"/>
       <c r="D65" s="14" t="s">
         <v>141</v>
       </c>
@@ -2738,9 +2741,9 @@
       <c r="F65" s="42"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="56"/>
-      <c r="B66" s="56"/>
-      <c r="C66" s="64"/>
+      <c r="A66" s="71"/>
+      <c r="B66" s="71"/>
+      <c r="C66" s="61"/>
       <c r="D66" s="14" t="s">
         <v>142</v>
       </c>
@@ -2750,9 +2753,9 @@
       <c r="F66" s="42"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="56"/>
-      <c r="B67" s="56"/>
-      <c r="C67" s="64"/>
+      <c r="A67" s="71"/>
+      <c r="B67" s="71"/>
+      <c r="C67" s="61"/>
       <c r="D67" s="14" t="s">
         <v>143</v>
       </c>
@@ -2762,9 +2765,9 @@
       <c r="F67" s="42"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="56"/>
-      <c r="B68" s="56"/>
-      <c r="C68" s="64"/>
+      <c r="A68" s="71"/>
+      <c r="B68" s="71"/>
+      <c r="C68" s="61"/>
       <c r="D68" s="14" t="s">
         <v>144</v>
       </c>
@@ -2774,9 +2777,9 @@
       <c r="F68" s="42"/>
     </row>
     <row r="69" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="57"/>
-      <c r="B69" s="57"/>
-      <c r="C69" s="65"/>
+      <c r="A69" s="72"/>
+      <c r="B69" s="72"/>
+      <c r="C69" s="62"/>
       <c r="D69" s="15" t="s">
         <v>145</v>
       </c>
@@ -2786,10 +2789,10 @@
       <c r="F69" s="42"/>
     </row>
     <row r="70" spans="1:6" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A70" s="66" t="s">
+      <c r="A70" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="B70" s="61" t="s">
+      <c r="B70" s="66" t="s">
         <v>39</v>
       </c>
       <c r="C70" s="63" t="s">
@@ -2804,9 +2807,9 @@
       <c r="F70" s="43"/>
     </row>
     <row r="71" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A71" s="67"/>
-      <c r="B71" s="62"/>
-      <c r="C71" s="64"/>
+      <c r="A71" s="65"/>
+      <c r="B71" s="60"/>
+      <c r="C71" s="61"/>
       <c r="D71" s="14" t="s">
         <v>79</v>
       </c>
@@ -2816,9 +2819,9 @@
       <c r="F71" s="44"/>
     </row>
     <row r="72" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A72" s="67"/>
-      <c r="B72" s="62"/>
-      <c r="C72" s="64"/>
+      <c r="A72" s="65"/>
+      <c r="B72" s="60"/>
+      <c r="C72" s="61"/>
       <c r="D72" s="14" t="s">
         <v>150</v>
       </c>
@@ -2827,10 +2830,10 @@
       </c>
       <c r="F72" s="44"/>
     </row>
-    <row r="73" spans="1:6" ht="51" x14ac:dyDescent="0.25">
-      <c r="A73" s="67"/>
-      <c r="B73" s="62"/>
-      <c r="C73" s="64"/>
+    <row r="73" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A73" s="65"/>
+      <c r="B73" s="60"/>
+      <c r="C73" s="61"/>
       <c r="D73" s="14" t="s">
         <v>151</v>
       </c>
@@ -2840,9 +2843,9 @@
       <c r="F73" s="44"/>
     </row>
     <row r="74" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="67"/>
-      <c r="B74" s="62"/>
-      <c r="C74" s="65"/>
+      <c r="A74" s="65"/>
+      <c r="B74" s="60"/>
+      <c r="C74" s="62"/>
       <c r="D74" s="14" t="s">
         <v>152</v>
       </c>
@@ -2870,10 +2873,10 @@
       <c r="F75" s="2"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="56" t="s">
+      <c r="A76" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="B76" s="56" t="s">
+      <c r="B76" s="71" t="s">
         <v>43</v>
       </c>
       <c r="C76" s="63" t="s">
@@ -2888,9 +2891,9 @@
       <c r="F76" s="37"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="56"/>
-      <c r="B77" s="56"/>
-      <c r="C77" s="64"/>
+      <c r="A77" s="71"/>
+      <c r="B77" s="71"/>
+      <c r="C77" s="61"/>
       <c r="D77" s="14" t="s">
         <v>45</v>
       </c>
@@ -2900,9 +2903,9 @@
       <c r="F77" s="38"/>
     </row>
     <row r="78" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A78" s="56"/>
-      <c r="B78" s="56"/>
-      <c r="C78" s="64"/>
+      <c r="A78" s="71"/>
+      <c r="B78" s="71"/>
+      <c r="C78" s="61"/>
       <c r="D78" s="14" t="s">
         <v>46</v>
       </c>
@@ -2912,9 +2915,9 @@
       <c r="F78" s="38"/>
     </row>
     <row r="79" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A79" s="56"/>
-      <c r="B79" s="56"/>
-      <c r="C79" s="64"/>
+      <c r="A79" s="71"/>
+      <c r="B79" s="71"/>
+      <c r="C79" s="61"/>
       <c r="D79" s="14" t="s">
         <v>47</v>
       </c>
@@ -2924,9 +2927,9 @@
       <c r="F79" s="38"/>
     </row>
     <row r="80" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="57"/>
-      <c r="B80" s="57"/>
-      <c r="C80" s="65"/>
+      <c r="A80" s="72"/>
+      <c r="B80" s="72"/>
+      <c r="C80" s="62"/>
       <c r="D80" s="15" t="s">
         <v>48</v>
       </c>
@@ -2936,16 +2939,16 @@
       <c r="F80" s="39"/>
     </row>
     <row r="81" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A81" s="55" t="s">
+      <c r="A81" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="B81" s="55" t="s">
+      <c r="B81" s="70" t="s">
         <v>50</v>
       </c>
       <c r="C81" s="63" t="s">
         <v>129</v>
       </c>
-      <c r="D81" s="61" t="s">
+      <c r="D81" s="66" t="s">
         <v>51</v>
       </c>
       <c r="E81" s="7" t="s">
@@ -2954,30 +2957,30 @@
       <c r="F81" s="37"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="56"/>
-      <c r="B82" s="56"/>
-      <c r="C82" s="64"/>
-      <c r="D82" s="62"/>
+      <c r="A82" s="71"/>
+      <c r="B82" s="71"/>
+      <c r="C82" s="61"/>
+      <c r="D82" s="60"/>
       <c r="E82" s="7" t="s">
         <v>155</v>
       </c>
       <c r="F82" s="38"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A83" s="56"/>
-      <c r="B83" s="56"/>
-      <c r="C83" s="64"/>
-      <c r="D83" s="62"/>
+      <c r="A83" s="71"/>
+      <c r="B83" s="71"/>
+      <c r="C83" s="61"/>
+      <c r="D83" s="60"/>
       <c r="E83" s="7" t="s">
         <v>156</v>
       </c>
       <c r="F83" s="38"/>
     </row>
     <row r="84" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A84" s="56"/>
-      <c r="B84" s="56"/>
-      <c r="C84" s="64"/>
-      <c r="D84" s="62" t="s">
+      <c r="A84" s="71"/>
+      <c r="B84" s="71"/>
+      <c r="C84" s="61"/>
+      <c r="D84" s="60" t="s">
         <v>52</v>
       </c>
       <c r="E84" s="7" t="s">
@@ -2986,30 +2989,30 @@
       <c r="F84" s="38"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" s="56"/>
-      <c r="B85" s="56"/>
-      <c r="C85" s="64"/>
-      <c r="D85" s="62"/>
+      <c r="A85" s="71"/>
+      <c r="B85" s="71"/>
+      <c r="C85" s="61"/>
+      <c r="D85" s="60"/>
       <c r="E85" s="7" t="s">
         <v>158</v>
       </c>
       <c r="F85" s="38"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" s="56"/>
-      <c r="B86" s="56"/>
-      <c r="C86" s="64"/>
-      <c r="D86" s="62"/>
+      <c r="A86" s="71"/>
+      <c r="B86" s="71"/>
+      <c r="C86" s="61"/>
+      <c r="D86" s="60"/>
       <c r="E86" s="7" t="s">
         <v>267</v>
       </c>
       <c r="F86" s="38"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" s="56"/>
-      <c r="B87" s="56"/>
-      <c r="C87" s="64"/>
-      <c r="D87" s="62" t="s">
+      <c r="A87" s="71"/>
+      <c r="B87" s="71"/>
+      <c r="C87" s="61"/>
+      <c r="D87" s="60" t="s">
         <v>53</v>
       </c>
       <c r="E87" s="7" t="s">
@@ -3018,30 +3021,30 @@
       <c r="F87" s="38"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" s="56"/>
-      <c r="B88" s="56"/>
-      <c r="C88" s="64"/>
-      <c r="D88" s="62"/>
+      <c r="A88" s="71"/>
+      <c r="B88" s="71"/>
+      <c r="C88" s="61"/>
+      <c r="D88" s="60"/>
       <c r="E88" s="7" t="s">
         <v>268</v>
       </c>
       <c r="F88" s="38"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" s="56"/>
-      <c r="B89" s="56"/>
-      <c r="C89" s="64"/>
-      <c r="D89" s="62"/>
+      <c r="A89" s="71"/>
+      <c r="B89" s="71"/>
+      <c r="C89" s="61"/>
+      <c r="D89" s="60"/>
       <c r="E89" s="7" t="s">
         <v>160</v>
       </c>
       <c r="F89" s="38"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" s="56"/>
-      <c r="B90" s="56"/>
-      <c r="C90" s="64"/>
-      <c r="D90" s="62" t="s">
+      <c r="A90" s="71"/>
+      <c r="B90" s="71"/>
+      <c r="C90" s="61"/>
+      <c r="D90" s="60" t="s">
         <v>54</v>
       </c>
       <c r="E90" s="7" t="s">
@@ -3050,30 +3053,30 @@
       <c r="F90" s="38"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A91" s="56"/>
-      <c r="B91" s="56"/>
-      <c r="C91" s="64"/>
-      <c r="D91" s="62"/>
+      <c r="A91" s="71"/>
+      <c r="B91" s="71"/>
+      <c r="C91" s="61"/>
+      <c r="D91" s="60"/>
       <c r="E91" s="7" t="s">
         <v>269</v>
       </c>
       <c r="F91" s="38"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A92" s="56"/>
-      <c r="B92" s="56"/>
-      <c r="C92" s="64"/>
-      <c r="D92" s="62"/>
+      <c r="A92" s="71"/>
+      <c r="B92" s="71"/>
+      <c r="C92" s="61"/>
+      <c r="D92" s="60"/>
       <c r="E92" s="7" t="s">
         <v>162</v>
       </c>
       <c r="F92" s="38"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" s="56"/>
-      <c r="B93" s="56"/>
-      <c r="C93" s="64"/>
-      <c r="D93" s="62" t="s">
+      <c r="A93" s="71"/>
+      <c r="B93" s="71"/>
+      <c r="C93" s="61"/>
+      <c r="D93" s="60" t="s">
         <v>55</v>
       </c>
       <c r="E93" s="7" t="s">
@@ -3082,30 +3085,30 @@
       <c r="F93" s="38"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A94" s="56"/>
-      <c r="B94" s="56"/>
-      <c r="C94" s="64"/>
-      <c r="D94" s="62"/>
+      <c r="A94" s="71"/>
+      <c r="B94" s="71"/>
+      <c r="C94" s="61"/>
+      <c r="D94" s="60"/>
       <c r="E94" s="7" t="s">
         <v>164</v>
       </c>
       <c r="F94" s="38"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A95" s="56"/>
-      <c r="B95" s="56"/>
-      <c r="C95" s="64"/>
-      <c r="D95" s="62"/>
+      <c r="A95" s="71"/>
+      <c r="B95" s="71"/>
+      <c r="C95" s="61"/>
+      <c r="D95" s="60"/>
       <c r="E95" s="7" t="s">
         <v>165</v>
       </c>
       <c r="F95" s="38"/>
     </row>
     <row r="96" spans="1:6" ht="51" x14ac:dyDescent="0.25">
-      <c r="A96" s="56"/>
-      <c r="B96" s="56"/>
-      <c r="C96" s="64"/>
-      <c r="D96" s="62" t="s">
+      <c r="A96" s="71"/>
+      <c r="B96" s="71"/>
+      <c r="C96" s="61"/>
+      <c r="D96" s="60" t="s">
         <v>153</v>
       </c>
       <c r="E96" s="7" t="s">
@@ -3114,30 +3117,30 @@
       <c r="F96" s="38"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" s="56"/>
-      <c r="B97" s="56"/>
-      <c r="C97" s="64"/>
-      <c r="D97" s="62"/>
+      <c r="A97" s="71"/>
+      <c r="B97" s="71"/>
+      <c r="C97" s="61"/>
+      <c r="D97" s="60"/>
       <c r="E97" s="7" t="s">
         <v>166</v>
       </c>
       <c r="F97" s="38"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" s="56"/>
-      <c r="B98" s="56"/>
-      <c r="C98" s="64"/>
-      <c r="D98" s="62"/>
+      <c r="A98" s="71"/>
+      <c r="B98" s="71"/>
+      <c r="C98" s="61"/>
+      <c r="D98" s="60"/>
       <c r="E98" s="7" t="s">
         <v>167</v>
       </c>
       <c r="F98" s="38"/>
     </row>
-    <row r="99" spans="1:6" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A99" s="56"/>
-      <c r="B99" s="56"/>
-      <c r="C99" s="64"/>
-      <c r="D99" s="62" t="s">
+    <row r="99" spans="1:6" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A99" s="71"/>
+      <c r="B99" s="71"/>
+      <c r="C99" s="61"/>
+      <c r="D99" s="60" t="s">
         <v>172</v>
       </c>
       <c r="E99" s="7" t="s">
@@ -3146,29 +3149,29 @@
       <c r="F99" s="38"/>
     </row>
     <row r="100" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A100" s="56"/>
-      <c r="B100" s="56"/>
-      <c r="C100" s="64"/>
-      <c r="D100" s="62"/>
+      <c r="A100" s="71"/>
+      <c r="B100" s="71"/>
+      <c r="C100" s="61"/>
+      <c r="D100" s="60"/>
       <c r="E100" s="7" t="s">
         <v>173</v>
       </c>
       <c r="F100" s="38"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A101" s="56"/>
-      <c r="B101" s="56"/>
-      <c r="C101" s="64"/>
-      <c r="D101" s="62"/>
+      <c r="A101" s="71"/>
+      <c r="B101" s="71"/>
+      <c r="C101" s="61"/>
+      <c r="D101" s="60"/>
       <c r="E101" s="7" t="s">
         <v>174</v>
       </c>
       <c r="F101" s="38"/>
     </row>
     <row r="102" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="57"/>
-      <c r="B102" s="57"/>
-      <c r="C102" s="65"/>
+      <c r="A102" s="72"/>
+      <c r="B102" s="72"/>
+      <c r="C102" s="62"/>
       <c r="D102" s="14" t="s">
         <v>48</v>
       </c>
@@ -3178,10 +3181,10 @@
       <c r="F102" s="39"/>
     </row>
     <row r="103" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A103" s="55" t="s">
+      <c r="A103" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="B103" s="55" t="s">
+      <c r="B103" s="70" t="s">
         <v>57</v>
       </c>
       <c r="C103" s="63" t="s">
@@ -3196,9 +3199,9 @@
       <c r="F103" s="37"/>
     </row>
     <row r="104" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A104" s="56"/>
-      <c r="B104" s="56"/>
-      <c r="C104" s="64"/>
+      <c r="A104" s="71"/>
+      <c r="B104" s="71"/>
+      <c r="C104" s="61"/>
       <c r="D104" s="32" t="s">
         <v>177</v>
       </c>
@@ -3208,9 +3211,9 @@
       <c r="F104" s="38"/>
     </row>
     <row r="105" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="57"/>
-      <c r="B105" s="57"/>
-      <c r="C105" s="65"/>
+      <c r="A105" s="72"/>
+      <c r="B105" s="72"/>
+      <c r="C105" s="62"/>
       <c r="D105" s="33" t="s">
         <v>180</v>
       </c>
@@ -3292,13 +3295,13 @@
       <c r="F109" s="4"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" s="55" t="s">
+      <c r="A110" s="70" t="s">
         <v>66</v>
       </c>
-      <c r="B110" s="55" t="s">
+      <c r="B110" s="70" t="s">
         <v>244</v>
       </c>
-      <c r="C110" s="64" t="s">
+      <c r="C110" s="61" t="s">
         <v>243</v>
       </c>
       <c r="D110" s="14" t="s">
@@ -3310,9 +3313,9 @@
       <c r="F110" s="37"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" s="56"/>
-      <c r="B111" s="56"/>
-      <c r="C111" s="64"/>
+      <c r="A111" s="71"/>
+      <c r="B111" s="71"/>
+      <c r="C111" s="61"/>
       <c r="D111" s="14" t="s">
         <v>68</v>
       </c>
@@ -3322,9 +3325,9 @@
       <c r="F111" s="38"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="56"/>
-      <c r="B112" s="56"/>
-      <c r="C112" s="64"/>
+      <c r="A112" s="71"/>
+      <c r="B112" s="71"/>
+      <c r="C112" s="61"/>
       <c r="D112" s="14" t="s">
         <v>69</v>
       </c>
@@ -3334,9 +3337,9 @@
       <c r="F112" s="38"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" s="56"/>
-      <c r="B113" s="56"/>
-      <c r="C113" s="64"/>
+      <c r="A113" s="71"/>
+      <c r="B113" s="71"/>
+      <c r="C113" s="61"/>
       <c r="D113" s="30" t="s">
         <v>181</v>
       </c>
@@ -3346,9 +3349,9 @@
       <c r="F113" s="38"/>
     </row>
     <row r="114" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="57"/>
-      <c r="B114" s="57"/>
-      <c r="C114" s="65"/>
+      <c r="A114" s="72"/>
+      <c r="B114" s="72"/>
+      <c r="C114" s="62"/>
       <c r="D114" s="15" t="s">
         <v>182</v>
       </c>
@@ -3376,10 +3379,10 @@
       <c r="F115" s="2"/>
     </row>
     <row r="116" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="58" t="s">
+      <c r="A116" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="B116" s="58" t="s">
+      <c r="B116" s="67" t="s">
         <v>73</v>
       </c>
       <c r="C116" s="63" t="s">
@@ -3394,9 +3397,9 @@
       <c r="F116" s="37"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A117" s="59"/>
-      <c r="B117" s="59"/>
-      <c r="C117" s="64"/>
+      <c r="A117" s="68"/>
+      <c r="B117" s="68"/>
+      <c r="C117" s="61"/>
       <c r="D117" s="47" t="s">
         <v>190</v>
       </c>
@@ -3406,9 +3409,9 @@
       <c r="F117" s="38"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A118" s="59"/>
-      <c r="B118" s="59"/>
-      <c r="C118" s="64"/>
+      <c r="A118" s="68"/>
+      <c r="B118" s="68"/>
+      <c r="C118" s="61"/>
       <c r="D118" s="47" t="s">
         <v>192</v>
       </c>
@@ -3418,9 +3421,9 @@
       <c r="F118" s="38"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A119" s="59"/>
-      <c r="B119" s="59"/>
-      <c r="C119" s="64"/>
+      <c r="A119" s="68"/>
+      <c r="B119" s="68"/>
+      <c r="C119" s="61"/>
       <c r="D119" s="47" t="s">
         <v>194</v>
       </c>
@@ -3430,9 +3433,9 @@
       <c r="F119" s="38"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A120" s="59"/>
-      <c r="B120" s="59"/>
-      <c r="C120" s="64"/>
+      <c r="A120" s="68"/>
+      <c r="B120" s="68"/>
+      <c r="C120" s="61"/>
       <c r="D120" s="47" t="s">
         <v>196</v>
       </c>
@@ -3442,9 +3445,9 @@
       <c r="F120" s="38"/>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A121" s="59"/>
-      <c r="B121" s="59"/>
-      <c r="C121" s="64"/>
+      <c r="A121" s="68"/>
+      <c r="B121" s="68"/>
+      <c r="C121" s="61"/>
       <c r="D121" s="47" t="s">
         <v>198</v>
       </c>
@@ -3454,9 +3457,9 @@
       <c r="F121" s="38"/>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A122" s="59"/>
-      <c r="B122" s="59"/>
-      <c r="C122" s="64"/>
+      <c r="A122" s="68"/>
+      <c r="B122" s="68"/>
+      <c r="C122" s="61"/>
       <c r="D122" s="47" t="s">
         <v>200</v>
       </c>
@@ -3466,9 +3469,9 @@
       <c r="F122" s="38"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A123" s="59"/>
-      <c r="B123" s="59"/>
-      <c r="C123" s="64"/>
+      <c r="A123" s="68"/>
+      <c r="B123" s="68"/>
+      <c r="C123" s="61"/>
       <c r="D123" s="47" t="s">
         <v>202</v>
       </c>
@@ -3478,9 +3481,9 @@
       <c r="F123" s="38"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A124" s="59"/>
-      <c r="B124" s="59"/>
-      <c r="C124" s="64"/>
+      <c r="A124" s="68"/>
+      <c r="B124" s="68"/>
+      <c r="C124" s="61"/>
       <c r="D124" s="47" t="s">
         <v>204</v>
       </c>
@@ -3490,9 +3493,9 @@
       <c r="F124" s="38"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A125" s="59"/>
-      <c r="B125" s="59"/>
-      <c r="C125" s="64"/>
+      <c r="A125" s="68"/>
+      <c r="B125" s="68"/>
+      <c r="C125" s="61"/>
       <c r="D125" s="47" t="s">
         <v>206</v>
       </c>
@@ -3502,9 +3505,9 @@
       <c r="F125" s="38"/>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A126" s="59"/>
-      <c r="B126" s="59"/>
-      <c r="C126" s="64"/>
+      <c r="A126" s="68"/>
+      <c r="B126" s="68"/>
+      <c r="C126" s="61"/>
       <c r="D126" s="47" t="s">
         <v>208</v>
       </c>
@@ -3514,9 +3517,9 @@
       <c r="F126" s="38"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A127" s="59"/>
-      <c r="B127" s="59"/>
-      <c r="C127" s="64"/>
+      <c r="A127" s="68"/>
+      <c r="B127" s="68"/>
+      <c r="C127" s="61"/>
       <c r="D127" s="47" t="s">
         <v>210</v>
       </c>
@@ -3526,9 +3529,9 @@
       <c r="F127" s="38"/>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A128" s="59"/>
-      <c r="B128" s="59"/>
-      <c r="C128" s="64"/>
+      <c r="A128" s="68"/>
+      <c r="B128" s="68"/>
+      <c r="C128" s="61"/>
       <c r="D128" s="47" t="s">
         <v>212</v>
       </c>
@@ -3538,9 +3541,9 @@
       <c r="F128" s="38"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A129" s="59"/>
-      <c r="B129" s="59"/>
-      <c r="C129" s="64"/>
+      <c r="A129" s="68"/>
+      <c r="B129" s="68"/>
+      <c r="C129" s="61"/>
       <c r="D129" s="47" t="s">
         <v>214</v>
       </c>
@@ -3550,9 +3553,9 @@
       <c r="F129" s="38"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A130" s="59"/>
-      <c r="B130" s="59"/>
-      <c r="C130" s="64"/>
+      <c r="A130" s="68"/>
+      <c r="B130" s="68"/>
+      <c r="C130" s="61"/>
       <c r="D130" s="47" t="s">
         <v>216</v>
       </c>
@@ -3562,9 +3565,9 @@
       <c r="F130" s="38"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A131" s="59"/>
-      <c r="B131" s="59"/>
-      <c r="C131" s="64"/>
+      <c r="A131" s="68"/>
+      <c r="B131" s="68"/>
+      <c r="C131" s="61"/>
       <c r="D131" s="47" t="s">
         <v>218</v>
       </c>
@@ -3574,9 +3577,9 @@
       <c r="F131" s="38"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A132" s="59"/>
-      <c r="B132" s="59"/>
-      <c r="C132" s="64"/>
+      <c r="A132" s="68"/>
+      <c r="B132" s="68"/>
+      <c r="C132" s="61"/>
       <c r="D132" s="47" t="s">
         <v>220</v>
       </c>
@@ -3586,9 +3589,9 @@
       <c r="F132" s="38"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A133" s="59"/>
-      <c r="B133" s="59"/>
-      <c r="C133" s="64"/>
+      <c r="A133" s="68"/>
+      <c r="B133" s="68"/>
+      <c r="C133" s="61"/>
       <c r="D133" s="47" t="s">
         <v>222</v>
       </c>
@@ -3598,9 +3601,9 @@
       <c r="F133" s="38"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A134" s="59"/>
-      <c r="B134" s="59"/>
-      <c r="C134" s="64"/>
+      <c r="A134" s="68"/>
+      <c r="B134" s="68"/>
+      <c r="C134" s="61"/>
       <c r="D134" s="47" t="s">
         <v>224</v>
       </c>
@@ -3610,9 +3613,9 @@
       <c r="F134" s="38"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A135" s="59"/>
-      <c r="B135" s="59"/>
-      <c r="C135" s="64"/>
+      <c r="A135" s="68"/>
+      <c r="B135" s="68"/>
+      <c r="C135" s="61"/>
       <c r="D135" s="47" t="s">
         <v>226</v>
       </c>
@@ -3622,9 +3625,9 @@
       <c r="F135" s="38"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A136" s="59"/>
-      <c r="B136" s="59"/>
-      <c r="C136" s="64"/>
+      <c r="A136" s="68"/>
+      <c r="B136" s="68"/>
+      <c r="C136" s="61"/>
       <c r="D136" s="47" t="s">
         <v>228</v>
       </c>
@@ -3634,9 +3637,9 @@
       <c r="F136" s="38"/>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A137" s="59"/>
-      <c r="B137" s="59"/>
-      <c r="C137" s="64"/>
+      <c r="A137" s="68"/>
+      <c r="B137" s="68"/>
+      <c r="C137" s="61"/>
       <c r="D137" s="47" t="s">
         <v>228</v>
       </c>
@@ -3644,9 +3647,9 @@
       <c r="F137" s="38"/>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A138" s="59"/>
-      <c r="B138" s="59"/>
-      <c r="C138" s="64"/>
+      <c r="A138" s="68"/>
+      <c r="B138" s="68"/>
+      <c r="C138" s="61"/>
       <c r="D138" s="47" t="s">
         <v>230</v>
       </c>
@@ -3656,9 +3659,9 @@
       <c r="F138" s="38"/>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A139" s="59"/>
-      <c r="B139" s="59"/>
-      <c r="C139" s="64"/>
+      <c r="A139" s="68"/>
+      <c r="B139" s="68"/>
+      <c r="C139" s="61"/>
       <c r="D139" s="47" t="s">
         <v>232</v>
       </c>
@@ -3668,9 +3671,9 @@
       <c r="F139" s="38"/>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A140" s="59"/>
-      <c r="B140" s="59"/>
-      <c r="C140" s="64"/>
+      <c r="A140" s="68"/>
+      <c r="B140" s="68"/>
+      <c r="C140" s="61"/>
       <c r="D140" s="47" t="s">
         <v>234</v>
       </c>
@@ -3680,9 +3683,9 @@
       <c r="F140" s="38"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A141" s="59"/>
-      <c r="B141" s="59"/>
-      <c r="C141" s="64"/>
+      <c r="A141" s="68"/>
+      <c r="B141" s="68"/>
+      <c r="C141" s="61"/>
       <c r="D141" s="47" t="s">
         <v>236</v>
       </c>
@@ -3692,9 +3695,9 @@
       <c r="F141" s="38"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A142" s="59"/>
-      <c r="B142" s="59"/>
-      <c r="C142" s="64"/>
+      <c r="A142" s="68"/>
+      <c r="B142" s="68"/>
+      <c r="C142" s="61"/>
       <c r="D142" s="47" t="s">
         <v>238</v>
       </c>
@@ -3704,9 +3707,9 @@
       <c r="F142" s="38"/>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A143" s="59"/>
-      <c r="B143" s="59"/>
-      <c r="C143" s="64"/>
+      <c r="A143" s="68"/>
+      <c r="B143" s="68"/>
+      <c r="C143" s="61"/>
       <c r="D143" s="34" t="s">
         <v>74</v>
       </c>
@@ -3716,9 +3719,9 @@
       <c r="F143" s="38"/>
     </row>
     <row r="144" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="60"/>
-      <c r="B144" s="60"/>
-      <c r="C144" s="65"/>
+      <c r="A144" s="69"/>
+      <c r="B144" s="69"/>
+      <c r="C144" s="62"/>
       <c r="D144" s="49" t="s">
         <v>75</v>
       </c>
@@ -3746,7 +3749,35 @@
       <c r="F145" s="3"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{E11F5BF0-69CA-44BB-85F3-E3ED603EB111}"/>
   <mergeCells count="43">
+    <mergeCell ref="C116:C144"/>
+    <mergeCell ref="C103:C105"/>
+    <mergeCell ref="C110:C114"/>
+    <mergeCell ref="A4:A13"/>
+    <mergeCell ref="B4:B13"/>
+    <mergeCell ref="B35:B51"/>
+    <mergeCell ref="A35:A51"/>
+    <mergeCell ref="A52:A61"/>
+    <mergeCell ref="B52:B61"/>
+    <mergeCell ref="A62:A69"/>
+    <mergeCell ref="B62:B69"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="A19:A32"/>
+    <mergeCell ref="B19:B32"/>
+    <mergeCell ref="A70:A74"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="A116:A144"/>
+    <mergeCell ref="B116:B144"/>
+    <mergeCell ref="A110:A114"/>
+    <mergeCell ref="B110:B114"/>
+    <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="A81:A102"/>
+    <mergeCell ref="B81:B102"/>
     <mergeCell ref="D99:D101"/>
     <mergeCell ref="C4:C13"/>
     <mergeCell ref="C14:C18"/>
@@ -3762,34 +3793,7 @@
     <mergeCell ref="D90:D92"/>
     <mergeCell ref="D93:D95"/>
     <mergeCell ref="D96:D98"/>
-    <mergeCell ref="A70:A74"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="A116:A144"/>
-    <mergeCell ref="B116:B144"/>
-    <mergeCell ref="A110:A114"/>
-    <mergeCell ref="B110:B114"/>
-    <mergeCell ref="A103:A105"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="A81:A102"/>
-    <mergeCell ref="B81:B102"/>
-    <mergeCell ref="C116:C144"/>
-    <mergeCell ref="C103:C105"/>
-    <mergeCell ref="C110:C114"/>
-    <mergeCell ref="A4:A13"/>
-    <mergeCell ref="B4:B13"/>
-    <mergeCell ref="B35:B51"/>
     <mergeCell ref="D81:D83"/>
-    <mergeCell ref="A35:A51"/>
-    <mergeCell ref="A52:A61"/>
-    <mergeCell ref="B52:B61"/>
-    <mergeCell ref="A62:A69"/>
-    <mergeCell ref="B62:B69"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="A19:A32"/>
-    <mergeCell ref="B19:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>